<commit_message>
Recalibrate operating model to Geoff's 7/6 census plan
New census: full panel migrates wks 1-2 (~24-25 open), +1.7/mo M1-2 (27.4 end M2),
+4-6 across M3-4 (32.4 end M4), +3-5 across M5-6 (35.0 end M6), then to 50 by M24
and 56 by M36. Back-solved weekly/monthly admissions (end-census dev 0.01);
capacity hires re-timed to new ADC triggers (2nd CNA M2, 3rd RN M4, 3rd CNA M5,
4th RN M11...); IDG conversions/quality hires pulled forward (SW M6, LVN M8,
chaplain M10, QAPI M8, intake M10, volunteer M12); med dir 2 at M18. Added SBA
proceeds row to Weekly Cash. QA 15/15 (trough band asserted as known finding).

Results: FY EBITDA 575K/581K/866K; M12 cash 382K. FINDING: with the 30-day CHOW
hold the Aug trough is now -8.1K (was +5.5K at the old census) - faster growth
consumes cash in the hold window; deferral (+5.7K) or SBA-in-Aug (+89K) covers it;
60-day hold needs SBA/backstop (-129K unlevered).

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/financial_models/output/Azalea_Refuge_Operating_Model.xlsx
+++ b/financial_models/output/Azalea_Refuge_Operating_Model.xlsx
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -1747,43 +1747,43 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>6.5</v>
+        <v>12</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>4.55</v>
+        <v>8.02</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>4.9</v>
+        <v>5.62</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>3.74</v>
+        <v>4.26</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>2.45</v>
+        <v>2.76</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>2.34</v>
+        <v>2.61</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>2.4</v>
+        <v>2.65</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>2.47</v>
+        <v>2.68</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>2.44</v>
+        <v>2.61</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>2.2</v>
+        <v>3.04</v>
       </c>
       <c r="M6" s="7" t="n">
-        <v>2.24</v>
+        <v>3</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>2.17</v>
+        <v>3.05</v>
       </c>
       <c r="O6" s="7" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="7">
@@ -2405,67 +2405,67 @@
         <v/>
       </c>
       <c r="F16" s="7" t="n">
-        <v>8.1</v>
+        <v>13.58</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8.43</v>
+        <v>13.31</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>8.6</v>
+        <v>13.79</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>8.619999999999999</v>
+        <v>13.78</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>8.69</v>
+        <v>14.17</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>8.76</v>
+        <v>14.41</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>8.94</v>
+        <v>14.7</v>
       </c>
       <c r="M16" s="7" t="n">
-        <v>8.949999999999999</v>
+        <v>15.1</v>
       </c>
       <c r="N16" s="7" t="n">
-        <v>9.02</v>
+        <v>15.33</v>
       </c>
       <c r="O16" s="7" t="n">
-        <v>11.06</v>
+        <v>15.63</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>11.87</v>
+        <v>16.03</v>
       </c>
       <c r="Q16" s="7" t="n">
-        <v>12.67</v>
+        <v>16.26</v>
       </c>
       <c r="R16" s="7" t="n">
-        <v>13.47</v>
+        <v>16.56</v>
       </c>
       <c r="S16" s="7" t="n">
-        <v>14.28</v>
+        <v>16.95</v>
       </c>
       <c r="T16" s="7" t="n">
-        <v>15.08</v>
+        <v>17.19</v>
       </c>
       <c r="U16" s="7" t="n">
-        <v>15.88</v>
+        <v>17.48</v>
       </c>
       <c r="V16" s="7" t="n">
-        <v>16.69</v>
+        <v>17.88</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>17.49</v>
+        <v>18.11</v>
       </c>
       <c r="X16" s="7" t="n">
-        <v>18.29</v>
+        <v>18.41</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>19.1</v>
+        <v>18.81</v>
       </c>
       <c r="Z16" s="7" t="n">
-        <v>19.9</v>
+        <v>19.04</v>
       </c>
       <c r="AA16" s="7" t="n">
         <v>19.04</v>
@@ -6347,7 +6347,7 @@
         <v>46511</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="D13" s="25" t="inlineStr">
         <is>
@@ -6520,7 +6520,7 @@
         <v>58000</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D14" s="25" t="inlineStr">
         <is>
@@ -6693,7 +6693,7 @@
         <v>52000</v>
       </c>
       <c r="C15" s="8" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D15" s="25" t="inlineStr">
         <is>
@@ -6866,7 +6866,7 @@
         <v>55000</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="D16" s="25" t="inlineStr">
         <is>
@@ -7039,7 +7039,7 @@
         <v>76256</v>
       </c>
       <c r="C17" s="8" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="D17" s="25" t="inlineStr">
         <is>
@@ -7212,7 +7212,7 @@
         <v>46511</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="D18" s="25" t="inlineStr">
         <is>
@@ -7385,7 +7385,7 @@
         <v>76256</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D19" s="25" t="inlineStr">
         <is>
@@ -7558,7 +7558,7 @@
         <v>46511</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
@@ -7731,7 +7731,7 @@
         <v>76256</v>
       </c>
       <c r="C21" s="8" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
@@ -7904,7 +7904,7 @@
         <v>46511</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D22" s="25" t="inlineStr">
         <is>
@@ -8077,7 +8077,7 @@
         <v>46511</v>
       </c>
       <c r="C23" s="8" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
@@ -8250,7 +8250,7 @@
         <v>76256</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D24" s="25" t="inlineStr">
         <is>
@@ -8423,7 +8423,7 @@
         <v>80000</v>
       </c>
       <c r="C25" s="8" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D25" s="25" t="inlineStr">
         <is>
@@ -8596,7 +8596,7 @@
         <v>55000</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D26" s="25" t="inlineStr">
         <is>
@@ -8769,7 +8769,7 @@
         <v>50000</v>
       </c>
       <c r="C27" s="8" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D27" s="25" t="inlineStr">
         <is>
@@ -15567,7 +15567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16023,66 +16023,125 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>SBA proceeds (if toggled, lands 1st week of funding month)</t>
+        </is>
+      </c>
+      <c r="C11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,1=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,1=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,1=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,2=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,2=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,2=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,3=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,3=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,3=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,4=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,4=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,4=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,5=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,5=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,5=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,6=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,6=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,6=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="I11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,7=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,7=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,7=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="J11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,8=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,8=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,8=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,9=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,9=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,9=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,10=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,10=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,10=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="M11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,11=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,11=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,11=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,12=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,12=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,12=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+      <c r="O11" s="22">
+        <f>IF(OR(AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=1,13=1),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=2,13=5),AND('Assumptions'!$B$81=1,'Assumptions'!$B$82=3,13=10)),'Assumptions'!$B$83,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>ENDING CASH</t>
         </is>
       </c>
-      <c r="C11" s="23">
-        <f>'Assumptions'!$B$88+C5+C6+C7+C8+C9+C10</f>
-        <v/>
-      </c>
-      <c r="D11" s="23">
-        <f>C11+D5+D6+D7+D8+D9+D10</f>
-        <v/>
-      </c>
-      <c r="E11" s="23">
-        <f>D11+E5+E6+E7+E8+E9+E10</f>
-        <v/>
-      </c>
-      <c r="F11" s="23">
-        <f>E11+F5+F6+F7+F8+F9+F10</f>
-        <v/>
-      </c>
-      <c r="G11" s="23">
-        <f>F11+G5+G6+G7+G8+G9+G10</f>
-        <v/>
-      </c>
-      <c r="H11" s="23">
-        <f>G11+H5+H6+H7+H8+H9+H10</f>
-        <v/>
-      </c>
-      <c r="I11" s="23">
-        <f>H11+I5+I6+I7+I8+I9+I10</f>
-        <v/>
-      </c>
-      <c r="J11" s="23">
-        <f>I11+J5+J6+J7+J8+J9+J10</f>
-        <v/>
-      </c>
-      <c r="K11" s="23">
-        <f>J11+K5+K6+K7+K8+K9+K10</f>
-        <v/>
-      </c>
-      <c r="L11" s="23">
-        <f>K11+L5+L6+L7+L8+L9+L10</f>
-        <v/>
-      </c>
-      <c r="M11" s="23">
-        <f>L11+M5+M6+M7+M8+M9+M10</f>
-        <v/>
-      </c>
-      <c r="N11" s="23">
-        <f>M11+N5+N6+N7+N8+N9+N10</f>
-        <v/>
-      </c>
-      <c r="O11" s="23">
-        <f>N11+O5+O6+O7+O8+O9+O10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="C12" s="23">
+        <f>'Assumptions'!$B$88+C5+C6+C7+C8+C9+C10+C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="23">
+        <f>C12+D5+D6+D7+D8+D9+D10+D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="23">
+        <f>D12+E5+E6+E7+E8+E9+E10+E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="23">
+        <f>E12+F5+F6+F7+F8+F9+F10+F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="23">
+        <f>F12+G5+G6+G7+G8+G9+G10+G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="23">
+        <f>G12+H5+H6+H7+H8+H9+H10+H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="23">
+        <f>H12+I5+I6+I7+I8+I9+I10+I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="23">
+        <f>I12+J5+J6+J7+J8+J9+J10+J11</f>
+        <v/>
+      </c>
+      <c r="K12" s="23">
+        <f>J12+K5+K6+K7+K8+K9+K10+K11</f>
+        <v/>
+      </c>
+      <c r="L12" s="23">
+        <f>K12+L5+L6+L7+L8+L9+L10+L11</f>
+        <v/>
+      </c>
+      <c r="M12" s="23">
+        <f>L12+M5+M6+M7+M8+M9+M10+M11</f>
+        <v/>
+      </c>
+      <c r="N12" s="23">
+        <f>M12+N5+N6+N7+N8+N9+N10+N11</f>
+        <v/>
+      </c>
+      <c r="O12" s="23">
+        <f>N12+O5+O6+O7+O8+O9+O10+O11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Note: weekly receipts spread each month's collections evenly across its weeks; payroll halves on the 15th/EOM; vendor hits per the Assumptions bill calendar. Precision is operational, not accounting-grade.</t>
         </is>
@@ -16093,7 +16152,7 @@
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="C11:O11">
+  <conditionalFormatting sqref="C12:O12">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>'Assumptions'!$B$89</formula>
     </cfRule>

</xml_diff>